<commit_message>
feat: implement audit logging service and add core administrative and estimate management modules
</commit_message>
<xml_diff>
--- a/sample users.xlsx
+++ b/sample users.xlsx
@@ -356,7 +356,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -372,7 +372,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Verdana"/>
       <family val="2"/>
     </font>
@@ -383,20 +383,13 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Verdana"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Verdana"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Verdana"/>
@@ -468,40 +461,40 @@
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
@@ -510,17 +503,17 @@
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
-    </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -828,21 +821,21 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="21" width="7.147857142857143" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="22" width="28.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="23" width="28.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="22" width="28.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="22" width="24.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="23" width="20.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="23" width="16.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="22" width="22.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="23" width="21.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="22" width="29.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="22" width="23.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="23" width="18.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="22" width="32.71928571428572" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="23" width="32.71928571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="8" width="28.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="22" width="28.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="8" width="28.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="8" width="24.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="22" width="20.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="22" width="16.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="8" width="22.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="22" width="21.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="8" width="29.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="8" width="23.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="22" width="18.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="8" width="32.71928571428572" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="22" width="32.71928571428572" customWidth="1" bestFit="1"/>
     <col min="15" max="15" style="8" width="50.71928571428572" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="7" width="19.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="23" width="19.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="20.25">
@@ -1423,7 +1416,7 @@
       </c>
       <c r="P12" s="19"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="16.5">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
       <c r="A13" s="17">
         <v>62</v>
       </c>
@@ -1471,7 +1464,7 @@
       </c>
       <c r="P13" s="19"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="16.5">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
       <c r="A14" s="17">
         <v>63</v>
       </c>
@@ -1519,7 +1512,7 @@
       </c>
       <c r="P14" s="19"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="16.5">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
       <c r="A15" s="17">
         <v>64</v>
       </c>
@@ -1567,7 +1560,7 @@
       </c>
       <c r="P15" s="19"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="16.5">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
       <c r="A16" s="17">
         <v>65</v>
       </c>
@@ -1615,7 +1608,7 @@
       </c>
       <c r="P16" s="19"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="16.5">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
       <c r="A17" s="17">
         <v>66</v>
       </c>

</xml_diff>

<commit_message>
feat: implement estimate version control, scrutiny remarks trail, visual diff engine and role-based jurisdiction synchronization
</commit_message>
<xml_diff>
--- a/sample users.xlsx
+++ b/sample users.xlsx
@@ -356,7 +356,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -374,12 +374,6 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Verdana"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
@@ -444,7 +438,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -473,25 +467,22 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
@@ -503,7 +494,7 @@
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -820,82 +811,82 @@
   <dimension ref="A1:P25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="21" width="7.147857142857143" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="20" width="7.147857142857143" customWidth="1" bestFit="1"/>
     <col min="2" max="2" style="8" width="28.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="22" width="28.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="21" width="28.862142857142857" customWidth="1" bestFit="1"/>
     <col min="4" max="4" style="8" width="28.862142857142857" customWidth="1" bestFit="1"/>
     <col min="5" max="5" style="8" width="24.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="22" width="20.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="22" width="16.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="21" width="20.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="21" width="16.290714285714284" customWidth="1" bestFit="1"/>
     <col min="8" max="8" style="8" width="22.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="22" width="21.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="21" width="21.290714285714284" customWidth="1" bestFit="1"/>
     <col min="10" max="10" style="8" width="29.719285714285714" customWidth="1" bestFit="1"/>
     <col min="11" max="11" style="8" width="23.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="22" width="18.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="21" width="18.576428571428572" customWidth="1" bestFit="1"/>
     <col min="13" max="13" style="8" width="32.71928571428572" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="22" width="32.71928571428572" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="21" width="32.71928571428572" customWidth="1" bestFit="1"/>
     <col min="15" max="15" style="8" width="50.71928571428572" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="23" width="19.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="22" width="19.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="20.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="F1" s="14" t="s">
+      <c r="F1" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="G1" s="14" t="s">
+      <c r="G1" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="H1" s="15" t="s">
+      <c r="H1" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="I1" s="14" t="s">
+      <c r="I1" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="J1" s="13" t="s">
+      <c r="J1" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="K1" s="13" t="s">
+      <c r="K1" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="L1" s="14" t="s">
+      <c r="L1" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="M1" s="13" t="s">
+      <c r="M1" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="N1" s="14" t="s">
+      <c r="N1" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="O1" s="13" t="s">
+      <c r="O1" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="P1" s="16" t="s">
+      <c r="P1" s="15" t="s">
         <v>62</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
-      <c r="A2" s="17">
+      <c r="A2" s="16">
         <v>51</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C2" s="18">
+      <c r="C2" s="17">
         <v>9989999753</v>
       </c>
       <c r="D2" s="4" t="s">
@@ -904,16 +895,16 @@
       <c r="E2" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="F2" s="18">
+      <c r="F2" s="17">
         <v>9989989507</v>
       </c>
-      <c r="G2" s="18">
+      <c r="G2" s="17">
         <v>5</v>
       </c>
       <c r="H2" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="I2" s="18">
+      <c r="I2" s="17">
         <v>9989994708</v>
       </c>
       <c r="J2" s="4" t="s">
@@ -922,28 +913,28 @@
       <c r="K2" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="L2" s="18">
+      <c r="L2" s="17">
         <v>7331185790</v>
       </c>
       <c r="M2" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="N2" s="18">
+      <c r="N2" s="17">
         <v>7331185790</v>
       </c>
       <c r="O2" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="P2" s="19"/>
+      <c r="P2" s="18"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
-      <c r="A3" s="17">
+      <c r="A3" s="16">
         <v>52</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C3" s="18">
+      <c r="C3" s="17">
         <v>9989999753</v>
       </c>
       <c r="D3" s="4" t="s">
@@ -952,16 +943,16 @@
       <c r="E3" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="F3" s="18">
+      <c r="F3" s="17">
         <v>9989989507</v>
       </c>
-      <c r="G3" s="18">
+      <c r="G3" s="17">
         <v>5</v>
       </c>
       <c r="H3" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="I3" s="18">
+      <c r="I3" s="17">
         <v>9989994708</v>
       </c>
       <c r="J3" s="4" t="s">
@@ -970,28 +961,28 @@
       <c r="K3" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="L3" s="18">
+      <c r="L3" s="17">
         <v>7331185790</v>
       </c>
       <c r="M3" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="N3" s="18">
+      <c r="N3" s="17">
         <v>7995010496</v>
       </c>
       <c r="O3" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="P3" s="19"/>
+      <c r="P3" s="18"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
-      <c r="A4" s="17">
+      <c r="A4" s="16">
         <v>53</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C4" s="18">
+      <c r="C4" s="17">
         <v>9989999753</v>
       </c>
       <c r="D4" s="4" t="s">
@@ -1000,16 +991,16 @@
       <c r="E4" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="F4" s="18">
+      <c r="F4" s="17">
         <v>9989989507</v>
       </c>
-      <c r="G4" s="18">
+      <c r="G4" s="17">
         <v>5</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="I4" s="18">
+      <c r="I4" s="17">
         <v>9989994708</v>
       </c>
       <c r="J4" s="4" t="s">
@@ -1018,28 +1009,28 @@
       <c r="K4" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="L4" s="18">
+      <c r="L4" s="17">
         <v>7331185790</v>
       </c>
       <c r="M4" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="N4" s="18">
+      <c r="N4" s="17">
         <v>9154866620</v>
       </c>
       <c r="O4" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="P4" s="19"/>
+      <c r="P4" s="18"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
-      <c r="A5" s="17">
+      <c r="A5" s="16">
         <v>54</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C5" s="18">
+      <c r="C5" s="17">
         <v>9989999753</v>
       </c>
       <c r="D5" s="4" t="s">
@@ -1048,16 +1039,16 @@
       <c r="E5" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="F5" s="18">
+      <c r="F5" s="17">
         <v>9989989507</v>
       </c>
-      <c r="G5" s="18">
+      <c r="G5" s="17">
         <v>5</v>
       </c>
       <c r="H5" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="I5" s="18">
+      <c r="I5" s="17">
         <v>9989994708</v>
       </c>
       <c r="J5" s="4" t="s">
@@ -1066,28 +1057,28 @@
       <c r="K5" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="L5" s="18">
+      <c r="L5" s="17">
         <v>7331185790</v>
       </c>
       <c r="M5" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="N5" s="18">
+      <c r="N5" s="17">
         <v>9154866620</v>
       </c>
       <c r="O5" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="P5" s="19"/>
+      <c r="P5" s="18"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
-      <c r="A6" s="17">
+      <c r="A6" s="16">
         <v>55</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C6" s="18">
+      <c r="C6" s="17">
         <v>9989999753</v>
       </c>
       <c r="D6" s="4" t="s">
@@ -1096,16 +1087,16 @@
       <c r="E6" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="F6" s="18">
+      <c r="F6" s="17">
         <v>9989989507</v>
       </c>
-      <c r="G6" s="18">
+      <c r="G6" s="17">
         <v>5</v>
       </c>
       <c r="H6" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="I6" s="18">
+      <c r="I6" s="17">
         <v>9989994708</v>
       </c>
       <c r="J6" s="4" t="s">
@@ -1114,28 +1105,28 @@
       <c r="K6" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="L6" s="18">
+      <c r="L6" s="17">
         <v>7331185790</v>
       </c>
       <c r="M6" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="N6" s="18">
+      <c r="N6" s="17">
         <v>7995010510</v>
       </c>
       <c r="O6" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="P6" s="19"/>
+      <c r="P6" s="18"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
-      <c r="A7" s="17">
+      <c r="A7" s="16">
         <v>56</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C7" s="18">
+      <c r="C7" s="17">
         <v>9989999753</v>
       </c>
       <c r="D7" s="4" t="s">
@@ -1144,16 +1135,16 @@
       <c r="E7" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="F7" s="18">
+      <c r="F7" s="17">
         <v>9989989507</v>
       </c>
-      <c r="G7" s="18">
+      <c r="G7" s="17">
         <v>5</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="I7" s="18">
+      <c r="I7" s="17">
         <v>9989994708</v>
       </c>
       <c r="J7" s="4" t="s">
@@ -1162,28 +1153,28 @@
       <c r="K7" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="L7" s="18">
+      <c r="L7" s="17">
         <v>7331185790</v>
       </c>
       <c r="M7" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="N7" s="18">
+      <c r="N7" s="17">
         <v>7995010510</v>
       </c>
       <c r="O7" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="P7" s="19"/>
+      <c r="P7" s="18"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
-      <c r="A8" s="17">
+      <c r="A8" s="16">
         <v>57</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C8" s="18">
+      <c r="C8" s="17">
         <v>9989999753</v>
       </c>
       <c r="D8" s="4" t="s">
@@ -1192,16 +1183,16 @@
       <c r="E8" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="F8" s="18">
+      <c r="F8" s="17">
         <v>9989989507</v>
       </c>
-      <c r="G8" s="18">
+      <c r="G8" s="17">
         <v>5</v>
       </c>
       <c r="H8" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="I8" s="18">
+      <c r="I8" s="17">
         <v>9989994708</v>
       </c>
       <c r="J8" s="4" t="s">
@@ -1210,28 +1201,28 @@
       <c r="K8" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="L8" s="18">
+      <c r="L8" s="17">
         <v>7331185782</v>
       </c>
       <c r="M8" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="N8" s="18">
+      <c r="N8" s="17">
         <v>9154866700</v>
       </c>
       <c r="O8" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="P8" s="19"/>
+      <c r="P8" s="18"/>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
-      <c r="A9" s="17">
+      <c r="A9" s="16">
         <v>58</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C9" s="18">
+      <c r="C9" s="17">
         <v>9989999753</v>
       </c>
       <c r="D9" s="4" t="s">
@@ -1240,16 +1231,16 @@
       <c r="E9" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="F9" s="18">
+      <c r="F9" s="17">
         <v>9989989507</v>
       </c>
-      <c r="G9" s="18">
+      <c r="G9" s="17">
         <v>5</v>
       </c>
       <c r="H9" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="I9" s="18">
+      <c r="I9" s="17">
         <v>9989994708</v>
       </c>
       <c r="J9" s="4" t="s">
@@ -1258,28 +1249,28 @@
       <c r="K9" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="L9" s="18">
+      <c r="L9" s="17">
         <v>7331185782</v>
       </c>
       <c r="M9" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="N9" s="18">
+      <c r="N9" s="17">
         <v>9154866700</v>
       </c>
       <c r="O9" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="P9" s="19"/>
+      <c r="P9" s="18"/>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
-      <c r="A10" s="17">
+      <c r="A10" s="16">
         <v>59</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C10" s="18">
+      <c r="C10" s="17">
         <v>9989999753</v>
       </c>
       <c r="D10" s="4" t="s">
@@ -1288,16 +1279,16 @@
       <c r="E10" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="F10" s="18">
+      <c r="F10" s="17">
         <v>9989989507</v>
       </c>
-      <c r="G10" s="18">
+      <c r="G10" s="17">
         <v>5</v>
       </c>
       <c r="H10" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="I10" s="18">
+      <c r="I10" s="17">
         <v>9989994708</v>
       </c>
       <c r="J10" s="4" t="s">
@@ -1306,28 +1297,28 @@
       <c r="K10" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="L10" s="18">
+      <c r="L10" s="17">
         <v>7331185782</v>
       </c>
       <c r="M10" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="N10" s="18">
+      <c r="N10" s="17">
         <v>9154866634</v>
       </c>
       <c r="O10" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="P10" s="19"/>
+      <c r="P10" s="18"/>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
-      <c r="A11" s="17">
+      <c r="A11" s="16">
         <v>60</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C11" s="18">
+      <c r="C11" s="17">
         <v>9989999753</v>
       </c>
       <c r="D11" s="4" t="s">
@@ -1336,16 +1327,16 @@
       <c r="E11" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="F11" s="18">
+      <c r="F11" s="17">
         <v>9989989507</v>
       </c>
-      <c r="G11" s="18">
+      <c r="G11" s="17">
         <v>5</v>
       </c>
       <c r="H11" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="I11" s="18">
+      <c r="I11" s="17">
         <v>9989994708</v>
       </c>
       <c r="J11" s="4" t="s">
@@ -1354,28 +1345,28 @@
       <c r="K11" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="L11" s="18">
+      <c r="L11" s="17">
         <v>7331185782</v>
       </c>
       <c r="M11" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="N11" s="18">
+      <c r="N11" s="17">
         <v>9154866634</v>
       </c>
       <c r="O11" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="P11" s="19"/>
+      <c r="P11" s="18"/>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
-      <c r="A12" s="17">
+      <c r="A12" s="16">
         <v>61</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C12" s="18">
+      <c r="C12" s="17">
         <v>9989999753</v>
       </c>
       <c r="D12" s="4" t="s">
@@ -1384,16 +1375,16 @@
       <c r="E12" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="F12" s="18">
+      <c r="F12" s="17">
         <v>9989989507</v>
       </c>
-      <c r="G12" s="18">
+      <c r="G12" s="17">
         <v>5</v>
       </c>
       <c r="H12" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="I12" s="18">
+      <c r="I12" s="17">
         <v>9989994708</v>
       </c>
       <c r="J12" s="4" t="s">
@@ -1402,28 +1393,28 @@
       <c r="K12" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="L12" s="18">
+      <c r="L12" s="17">
         <v>7331185782</v>
       </c>
       <c r="M12" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="N12" s="18">
+      <c r="N12" s="17">
         <v>9154297397</v>
       </c>
       <c r="O12" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="P12" s="19"/>
+      <c r="P12" s="18"/>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
-      <c r="A13" s="17">
+      <c r="A13" s="16">
         <v>62</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C13" s="18">
+      <c r="C13" s="17">
         <v>9989999753</v>
       </c>
       <c r="D13" s="4" t="s">
@@ -1432,16 +1423,16 @@
       <c r="E13" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="F13" s="18">
+      <c r="F13" s="17">
         <v>9989989507</v>
       </c>
-      <c r="G13" s="18">
+      <c r="G13" s="17">
         <v>5</v>
       </c>
       <c r="H13" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="I13" s="18">
+      <c r="I13" s="17">
         <v>9989994708</v>
       </c>
       <c r="J13" s="4" t="s">
@@ -1450,28 +1441,28 @@
       <c r="K13" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="L13" s="18">
+      <c r="L13" s="17">
         <v>7331185782</v>
       </c>
       <c r="M13" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="N13" s="18">
+      <c r="N13" s="17">
         <v>9154297397</v>
       </c>
       <c r="O13" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="P13" s="19"/>
+      <c r="P13" s="18"/>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
-      <c r="A14" s="17">
+      <c r="A14" s="16">
         <v>63</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C14" s="18">
+      <c r="C14" s="17">
         <v>9989999753</v>
       </c>
       <c r="D14" s="4" t="s">
@@ -1480,16 +1471,16 @@
       <c r="E14" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="F14" s="18">
+      <c r="F14" s="17">
         <v>9989989507</v>
       </c>
-      <c r="G14" s="18">
+      <c r="G14" s="17">
         <v>5</v>
       </c>
       <c r="H14" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="I14" s="18">
+      <c r="I14" s="17">
         <v>9989994708</v>
       </c>
       <c r="J14" s="4" t="s">
@@ -1498,28 +1489,28 @@
       <c r="K14" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="L14" s="18">
+      <c r="L14" s="17">
         <v>7331185782</v>
       </c>
       <c r="M14" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="N14" s="18">
+      <c r="N14" s="17">
         <v>7331185782</v>
       </c>
       <c r="O14" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="P14" s="19"/>
+      <c r="P14" s="18"/>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
-      <c r="A15" s="17">
+      <c r="A15" s="16">
         <v>64</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C15" s="18">
+      <c r="C15" s="17">
         <v>9989999753</v>
       </c>
       <c r="D15" s="4" t="s">
@@ -1528,16 +1519,16 @@
       <c r="E15" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="F15" s="18">
+      <c r="F15" s="17">
         <v>9989989507</v>
       </c>
-      <c r="G15" s="18">
+      <c r="G15" s="17">
         <v>6</v>
       </c>
       <c r="H15" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="I15" s="18">
+      <c r="I15" s="17">
         <v>9989994708</v>
       </c>
       <c r="J15" s="4" t="s">
@@ -1546,28 +1537,28 @@
       <c r="K15" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="L15" s="18">
+      <c r="L15" s="17">
         <v>9989996103</v>
       </c>
       <c r="M15" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="N15" s="18">
+      <c r="N15" s="17">
         <v>9989999546</v>
       </c>
       <c r="O15" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="P15" s="19"/>
+      <c r="P15" s="18"/>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
-      <c r="A16" s="17">
+      <c r="A16" s="16">
         <v>65</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C16" s="18">
+      <c r="C16" s="17">
         <v>9989999753</v>
       </c>
       <c r="D16" s="4" t="s">
@@ -1576,16 +1567,16 @@
       <c r="E16" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="F16" s="18">
+      <c r="F16" s="17">
         <v>9989989507</v>
       </c>
-      <c r="G16" s="18">
+      <c r="G16" s="17">
         <v>6</v>
       </c>
       <c r="H16" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="I16" s="18">
+      <c r="I16" s="17">
         <v>9989994708</v>
       </c>
       <c r="J16" s="4" t="s">
@@ -1594,28 +1585,28 @@
       <c r="K16" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="L16" s="18">
+      <c r="L16" s="17">
         <v>9989996103</v>
       </c>
       <c r="M16" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="N16" s="18">
+      <c r="N16" s="17">
         <v>9989999546</v>
       </c>
       <c r="O16" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="P16" s="19"/>
+      <c r="P16" s="18"/>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
-      <c r="A17" s="17">
+      <c r="A17" s="16">
         <v>66</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C17" s="18">
+      <c r="C17" s="17">
         <v>9989999753</v>
       </c>
       <c r="D17" s="4" t="s">
@@ -1624,16 +1615,16 @@
       <c r="E17" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="F17" s="18">
+      <c r="F17" s="17">
         <v>9989989507</v>
       </c>
-      <c r="G17" s="18">
+      <c r="G17" s="17">
         <v>6</v>
       </c>
       <c r="H17" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="I17" s="18">
+      <c r="I17" s="17">
         <v>9989994708</v>
       </c>
       <c r="J17" s="4" t="s">
@@ -1642,28 +1633,28 @@
       <c r="K17" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="L17" s="18">
+      <c r="L17" s="17">
         <v>9989996103</v>
       </c>
       <c r="M17" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="N17" s="18">
+      <c r="N17" s="17">
         <v>9154866671</v>
       </c>
       <c r="O17" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="P17" s="19"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="16.5">
-      <c r="A18" s="17">
+      <c r="P17" s="18"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
+      <c r="A18" s="16">
         <v>67</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C18" s="18">
+      <c r="C18" s="17">
         <v>9989999753</v>
       </c>
       <c r="D18" s="4" t="s">
@@ -1672,16 +1663,16 @@
       <c r="E18" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="F18" s="18">
+      <c r="F18" s="17">
         <v>9989989507</v>
       </c>
-      <c r="G18" s="18">
+      <c r="G18" s="17">
         <v>6</v>
       </c>
       <c r="H18" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="I18" s="18">
+      <c r="I18" s="17">
         <v>9989994708</v>
       </c>
       <c r="J18" s="4" t="s">
@@ -1690,28 +1681,28 @@
       <c r="K18" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="L18" s="18">
+      <c r="L18" s="17">
         <v>9989996103</v>
       </c>
       <c r="M18" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="N18" s="18">
+      <c r="N18" s="17">
         <v>9989996103</v>
       </c>
       <c r="O18" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="P18" s="19"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="16.5">
-      <c r="A19" s="17">
+      <c r="P18" s="18"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
+      <c r="A19" s="16">
         <v>68</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C19" s="18">
+      <c r="C19" s="17">
         <v>9989999753</v>
       </c>
       <c r="D19" s="4" t="s">
@@ -1720,16 +1711,16 @@
       <c r="E19" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="F19" s="18">
+      <c r="F19" s="17">
         <v>9989989507</v>
       </c>
-      <c r="G19" s="18">
+      <c r="G19" s="17">
         <v>6</v>
       </c>
       <c r="H19" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="I19" s="18">
+      <c r="I19" s="17">
         <v>9989994708</v>
       </c>
       <c r="J19" s="4" t="s">
@@ -1738,28 +1729,28 @@
       <c r="K19" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="L19" s="18">
+      <c r="L19" s="17">
         <v>9989996103</v>
       </c>
       <c r="M19" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="N19" s="18">
+      <c r="N19" s="17">
         <v>9154866671</v>
       </c>
       <c r="O19" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="P19" s="19"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="16.5">
-      <c r="A20" s="17">
+      <c r="P19" s="18"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5">
+      <c r="A20" s="16">
         <v>69</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C20" s="18">
+      <c r="C20" s="17">
         <v>9989999753</v>
       </c>
       <c r="D20" s="4" t="s">
@@ -1768,16 +1759,16 @@
       <c r="E20" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="F20" s="18">
+      <c r="F20" s="17">
         <v>9989989507</v>
       </c>
-      <c r="G20" s="18">
+      <c r="G20" s="17">
         <v>6</v>
       </c>
       <c r="H20" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="I20" s="18">
+      <c r="I20" s="17">
         <v>9989994708</v>
       </c>
       <c r="J20" s="4" t="s">
@@ -1786,28 +1777,28 @@
       <c r="K20" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="L20" s="18">
+      <c r="L20" s="17">
         <v>9989994369</v>
       </c>
       <c r="M20" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="N20" s="18">
+      <c r="N20" s="17">
         <v>9154866585</v>
       </c>
       <c r="O20" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="P20" s="19"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="16.5">
-      <c r="A21" s="17">
+      <c r="P20" s="18"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="19.5">
+      <c r="A21" s="16">
         <v>70</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C21" s="18">
+      <c r="C21" s="17">
         <v>9989999753</v>
       </c>
       <c r="D21" s="4" t="s">
@@ -1816,16 +1807,16 @@
       <c r="E21" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="F21" s="18">
+      <c r="F21" s="17">
         <v>9989989507</v>
       </c>
-      <c r="G21" s="18">
+      <c r="G21" s="17">
         <v>6</v>
       </c>
       <c r="H21" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="I21" s="18">
+      <c r="I21" s="17">
         <v>9989994708</v>
       </c>
       <c r="J21" s="4" t="s">
@@ -1834,28 +1825,28 @@
       <c r="K21" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="L21" s="18">
+      <c r="L21" s="17">
         <v>9989994369</v>
       </c>
       <c r="M21" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="N21" s="18">
+      <c r="N21" s="17">
         <v>9154866585</v>
       </c>
       <c r="O21" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="P21" s="19"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="16.5">
-      <c r="A22" s="17">
+      <c r="P21" s="18"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="19.5">
+      <c r="A22" s="16">
         <v>71</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C22" s="18">
+      <c r="C22" s="17">
         <v>9989999753</v>
       </c>
       <c r="D22" s="4" t="s">
@@ -1864,16 +1855,16 @@
       <c r="E22" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="F22" s="18">
+      <c r="F22" s="17">
         <v>9989989507</v>
       </c>
-      <c r="G22" s="18">
+      <c r="G22" s="17">
         <v>6</v>
       </c>
       <c r="H22" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="I22" s="18">
+      <c r="I22" s="17">
         <v>9989994708</v>
       </c>
       <c r="J22" s="4" t="s">
@@ -1882,28 +1873,28 @@
       <c r="K22" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="L22" s="18">
+      <c r="L22" s="17">
         <v>9989994369</v>
       </c>
       <c r="M22" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="N22" s="18">
+      <c r="N22" s="17">
         <v>9154866643</v>
       </c>
       <c r="O22" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="P22" s="19"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
-      <c r="A23" s="17">
+      <c r="P22" s="18"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="19.5">
+      <c r="A23" s="16">
         <v>72</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C23" s="18">
+      <c r="C23" s="17">
         <v>9989999753</v>
       </c>
       <c r="D23" s="4" t="s">
@@ -1912,16 +1903,16 @@
       <c r="E23" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="F23" s="18">
+      <c r="F23" s="17">
         <v>9989989507</v>
       </c>
-      <c r="G23" s="18">
+      <c r="G23" s="17">
         <v>6</v>
       </c>
       <c r="H23" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="I23" s="18">
+      <c r="I23" s="17">
         <v>9989994708</v>
       </c>
       <c r="J23" s="4" t="s">
@@ -1930,28 +1921,28 @@
       <c r="K23" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="L23" s="18">
+      <c r="L23" s="17">
         <v>9989994369</v>
       </c>
       <c r="M23" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="N23" s="18">
+      <c r="N23" s="17">
         <v>9154866643</v>
       </c>
       <c r="O23" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="P23" s="19"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="16.5">
-      <c r="A24" s="17">
+      <c r="P23" s="18"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="19.5">
+      <c r="A24" s="16">
         <v>73</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C24" s="18">
+      <c r="C24" s="17">
         <v>9989999753</v>
       </c>
       <c r="D24" s="4" t="s">
@@ -1960,16 +1951,16 @@
       <c r="E24" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="F24" s="18">
+      <c r="F24" s="17">
         <v>9989989507</v>
       </c>
-      <c r="G24" s="18">
+      <c r="G24" s="17">
         <v>6</v>
       </c>
       <c r="H24" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="I24" s="18">
+      <c r="I24" s="17">
         <v>9989994708</v>
       </c>
       <c r="J24" s="4" t="s">
@@ -1978,28 +1969,28 @@
       <c r="K24" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="L24" s="18">
+      <c r="L24" s="17">
         <v>9989994369</v>
       </c>
       <c r="M24" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="N24" s="18">
+      <c r="N24" s="17">
         <v>9154866717</v>
       </c>
-      <c r="O24" s="20" t="s">
+      <c r="O24" s="19" t="s">
         <v>108</v>
       </c>
-      <c r="P24" s="19"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="16.5">
-      <c r="A25" s="17">
+      <c r="P24" s="18"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="20.25">
+      <c r="A25" s="16">
         <v>74</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C25" s="18">
+      <c r="C25" s="17">
         <v>9989999753</v>
       </c>
       <c r="D25" s="4" t="s">
@@ -2008,16 +1999,16 @@
       <c r="E25" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="F25" s="18">
+      <c r="F25" s="17">
         <v>9989989507</v>
       </c>
-      <c r="G25" s="18">
+      <c r="G25" s="17">
         <v>6</v>
       </c>
       <c r="H25" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="I25" s="18">
+      <c r="I25" s="17">
         <v>9989994708</v>
       </c>
       <c r="J25" s="4" t="s">
@@ -2026,19 +2017,19 @@
       <c r="K25" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="L25" s="18">
+      <c r="L25" s="17">
         <v>9989994369</v>
       </c>
       <c r="M25" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="N25" s="18">
+      <c r="N25" s="17">
         <v>9989994369</v>
       </c>
       <c r="O25" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="P25" s="19"/>
+      <c r="P25" s="18"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2053,8 +2044,8 @@
   <dimension ref="A1:B28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="11" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="11" width="26.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="10" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="10" width="26.719285714285714" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -2066,210 +2057,210 @@
       <c r="B2" s="9"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="9" t="s">
         <v>49</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="10">
+      <c r="A4" s="9">
         <v>1</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="9">
         <v>12</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="10">
+      <c r="A5" s="9">
         <v>2</v>
       </c>
-      <c r="B5" s="10">
+      <c r="B5" s="9">
         <v>14</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="10">
+      <c r="A6" s="9">
         <v>3</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="9">
         <v>9</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
-      <c r="A7" s="10">
+      <c r="A7" s="9">
         <v>4</v>
       </c>
-      <c r="B7" s="10">
+      <c r="B7" s="9">
         <v>15</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
-      <c r="A8" s="10">
+      <c r="A8" s="9">
         <v>5</v>
       </c>
-      <c r="B8" s="10">
+      <c r="B8" s="9">
         <v>13</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
-      <c r="A9" s="10">
+      <c r="A9" s="9">
         <v>6</v>
       </c>
-      <c r="B9" s="10">
+      <c r="B9" s="9">
         <v>11</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
-      <c r="A10" s="10">
+      <c r="A10" s="9">
         <v>7</v>
       </c>
-      <c r="B10" s="10">
+      <c r="B10" s="9">
         <v>10</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
-      <c r="A11" s="10">
+      <c r="A11" s="9">
         <v>8</v>
       </c>
-      <c r="B11" s="10">
+      <c r="B11" s="9">
         <v>7</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
-      <c r="A12" s="10">
+      <c r="A12" s="9">
         <v>9</v>
       </c>
-      <c r="B12" s="10">
+      <c r="B12" s="9">
         <v>10</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
-      <c r="A13" s="10">
+      <c r="A13" s="9">
         <v>10</v>
       </c>
-      <c r="B13" s="10">
+      <c r="B13" s="9">
         <v>19</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
-      <c r="A14" s="10">
+      <c r="A14" s="9">
         <v>11</v>
       </c>
-      <c r="B14" s="10">
+      <c r="B14" s="9">
         <v>12</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
-      <c r="A15" s="10">
+      <c r="A15" s="9">
         <v>12</v>
       </c>
-      <c r="B15" s="10">
+      <c r="B15" s="9">
         <v>13</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
-      <c r="A16" s="10">
+      <c r="A16" s="9">
         <v>13</v>
       </c>
-      <c r="B16" s="10">
+      <c r="B16" s="9">
         <v>11</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
-      <c r="A17" s="10">
+      <c r="A17" s="9">
         <v>14</v>
       </c>
-      <c r="B17" s="10">
+      <c r="B17" s="9">
         <v>15</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
-      <c r="A18" s="10">
+      <c r="A18" s="9">
         <v>15</v>
       </c>
-      <c r="B18" s="10">
+      <c r="B18" s="9">
         <v>10</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
-      <c r="A19" s="10">
+      <c r="A19" s="9">
         <v>16</v>
       </c>
-      <c r="B19" s="10">
+      <c r="B19" s="9">
         <v>15</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
-      <c r="A20" s="10">
+      <c r="A20" s="9">
         <v>17</v>
       </c>
-      <c r="B20" s="10">
+      <c r="B20" s="9">
         <v>20</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
-      <c r="A21" s="10">
+      <c r="A21" s="9">
         <v>18</v>
       </c>
-      <c r="B21" s="10">
+      <c r="B21" s="9">
         <v>8</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
-      <c r="A22" s="10">
+      <c r="A22" s="9">
         <v>19</v>
       </c>
-      <c r="B22" s="10">
+      <c r="B22" s="9">
         <v>9</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
-      <c r="A23" s="10">
+      <c r="A23" s="9">
         <v>20</v>
       </c>
-      <c r="B23" s="10">
+      <c r="B23" s="9">
         <v>17</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
-      <c r="A24" s="10">
+      <c r="A24" s="9">
         <v>21</v>
       </c>
-      <c r="B24" s="10">
+      <c r="B24" s="9">
         <v>12</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
-      <c r="A25" s="10">
+      <c r="A25" s="9">
         <v>22</v>
       </c>
-      <c r="B25" s="10">
+      <c r="B25" s="9">
         <v>11</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
-      <c r="A26" s="10">
+      <c r="A26" s="9">
         <v>23</v>
       </c>
-      <c r="B26" s="10">
+      <c r="B26" s="9">
         <v>17</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
-      <c r="A27" s="10">
+      <c r="A27" s="9">
         <v>24</v>
       </c>
-      <c r="B27" s="10">
+      <c r="B27" s="9">
         <v>10</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
-      <c r="A28" s="10" t="s">
+      <c r="A28" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="B28" s="10">
+      <c r="B28" s="9">
         <v>300</v>
       </c>
     </row>

</xml_diff>